<commit_message>
Test include lcia profile
</commit_message>
<xml_diff>
--- a/data/Example/model_inputs/Input_data_example.xlsx
+++ b/data/Example/model_inputs/Input_data_example.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:101_{93367A34-0ECE-48D8-82EC-F57212DB67C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:101_{93367A34-0ECE-48D8-82EC-F57212DB67C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D95C25B0-C80E-4044-ABD0-2A5A066D974D}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data_base_case" sheetId="79" r:id="rId1"/>
@@ -2092,7 +2092,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="279">
   <si>
     <t>Red: Don't change the name without changing the Julia code</t>
   </si>
@@ -2809,9 +2809,6 @@
   </si>
   <si>
     <t>https://backend.orbit.dtu.dk/ws/portalfiles/portal/264043718/MarE_Fuel_LCOE_and_optimal_electricity_supply_strategies_for_P2X_plants.pdf</t>
-  </si>
-  <si>
-    <t>Investment (EUR/Capacity installed)2025 bench</t>
   </si>
   <si>
     <t>Water supply (desalination plant)</t>
@@ -3931,16 +3928,16 @@
         <v>108</v>
       </c>
       <c r="G1" s="49" t="s">
+        <v>260</v>
+      </c>
+      <c r="H1" s="49" t="s">
         <v>261</v>
-      </c>
-      <c r="H1" s="49" t="s">
-        <v>262</v>
       </c>
       <c r="I1" s="49" t="s">
         <v>120</v>
       </c>
       <c r="J1" s="50" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K1" s="126" t="s">
         <v>2</v>
@@ -3982,7 +3979,7 @@
         <v>140</v>
       </c>
       <c r="X1" s="52" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="Y1" s="52" t="s">
         <v>141</v>
@@ -4183,7 +4180,7 @@
         <v>Used (1 or 0)All</v>
       </c>
       <c r="G4" s="15" t="str">
-        <f t="shared" ref="G4:H4" si="17">G2&amp;G3</f>
+        <f t="shared" ref="G4:AA4" si="17">G2&amp;G3</f>
         <v>Capacity unitsAll</v>
       </c>
       <c r="H4" s="15" t="str">
@@ -4191,78 +4188,79 @@
         <v>Output unitsAll</v>
       </c>
       <c r="I4" s="15" t="str">
-        <f>I2&amp;I3</f>
+        <f t="shared" si="17"/>
         <v>Unit tagAll</v>
       </c>
       <c r="J4" s="15" t="str">
-        <f t="shared" ref="J4:O4" si="18">J2&amp;J3</f>
+        <f t="shared" si="17"/>
         <v>Yearly demand (output)All</v>
       </c>
-      <c r="K4" s="127" t="str">
-        <f t="shared" si="18"/>
+      <c r="K4" s="15" t="str">
+        <f t="shared" si="17"/>
         <v>Produced fromAll</v>
       </c>
       <c r="L4" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>El balanceAll</v>
       </c>
       <c r="M4" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>Heat balanceAll</v>
       </c>
       <c r="N4" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>H2 balanceAll</v>
       </c>
       <c r="O4" s="15" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>Max CapacityAll</v>
       </c>
       <c r="P4" s="15" t="str">
-        <f t="shared" ref="P4:U4" si="19">P2&amp;P3</f>
+        <f t="shared" si="17"/>
         <v>Fuel production rate (kg output/kg input)2025</v>
       </c>
       <c r="Q4" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>Heat generated (kWh/output)2025</v>
       </c>
       <c r="R4" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>Load min (% of max capacity)2025</v>
       </c>
       <c r="S4" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>Ramp up (% of capacity /h)2025</v>
       </c>
       <c r="T4" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>Ramp down (% of capacity /h)2025</v>
       </c>
       <c r="U4" s="15" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="17"/>
         <v>Electrical consumption (kWh/output)2025</v>
       </c>
-      <c r="V4" s="15" t="s">
-        <v>239</v>
+      <c r="V4" s="15" t="str">
+        <f t="shared" si="17"/>
+        <v>Investment (EUR/Capacity installed)2025</v>
       </c>
       <c r="W4" s="15" t="str">
-        <f t="shared" ref="W4:AA4" si="20">W2&amp;W3</f>
+        <f t="shared" si="17"/>
         <v>Fixed cost (EUR/Capacity installed/y)2025</v>
       </c>
       <c r="X4" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="17"/>
         <v>Variable cost (EUR/output)2025</v>
       </c>
       <c r="Y4" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="17"/>
         <v>Fuel selling price (EUR/output)2025</v>
       </c>
       <c r="Z4" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="17"/>
         <v>Fuel buying price (EUR/output)2025</v>
       </c>
       <c r="AA4" s="15" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="17"/>
         <v>Annuity factor2025</v>
       </c>
     </row>
@@ -4274,35 +4272,35 @@
         <v>10</v>
       </c>
       <c r="F5" s="8">
-        <f t="shared" ref="F5:O5" si="21">COLUMN(F2)-COLUMN($E$5)</f>
+        <f t="shared" ref="F5:O5" si="18">COLUMN(F2)-COLUMN($E$5)</f>
         <v>1</v>
       </c>
       <c r="G5" s="8">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>2</v>
       </c>
       <c r="H5" s="8">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>3</v>
       </c>
       <c r="I5" s="8">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>4</v>
       </c>
       <c r="J5" s="8">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>5</v>
       </c>
       <c r="K5" s="128">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>6</v>
       </c>
       <c r="L5" s="8">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>7</v>
       </c>
       <c r="M5" s="8">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>8</v>
       </c>
       <c r="N5" s="8">
@@ -4310,54 +4308,54 @@
         <v>9</v>
       </c>
       <c r="O5" s="8">
-        <f t="shared" si="21"/>
+        <f t="shared" si="18"/>
         <v>10</v>
       </c>
       <c r="P5" s="8">
-        <f t="shared" ref="P5:U5" si="22">COLUMN(P2)-COLUMN($E$5)</f>
+        <f t="shared" ref="P5:U5" si="19">COLUMN(P2)-COLUMN($E$5)</f>
         <v>11</v>
       </c>
       <c r="Q5" s="8">
-        <f t="shared" si="22"/>
+        <f t="shared" si="19"/>
         <v>12</v>
       </c>
       <c r="R5" s="8">
-        <f t="shared" si="22"/>
+        <f t="shared" si="19"/>
         <v>13</v>
       </c>
       <c r="S5" s="8">
-        <f t="shared" si="22"/>
+        <f t="shared" si="19"/>
         <v>14</v>
       </c>
       <c r="T5" s="8">
-        <f t="shared" si="22"/>
+        <f t="shared" si="19"/>
         <v>15</v>
       </c>
       <c r="U5" s="8">
-        <f t="shared" si="22"/>
+        <f t="shared" si="19"/>
         <v>16</v>
       </c>
       <c r="V5" s="8">
         <v>17</v>
       </c>
       <c r="W5" s="8">
-        <f t="shared" ref="W5:AA5" si="23">COLUMN(W2)-COLUMN($E$5)</f>
+        <f t="shared" ref="W5:AA5" si="20">COLUMN(W2)-COLUMN($E$5)</f>
         <v>18</v>
       </c>
       <c r="X5" s="8">
-        <f t="shared" si="23"/>
+        <f t="shared" si="20"/>
         <v>19</v>
       </c>
       <c r="Y5" s="8">
-        <f t="shared" si="23"/>
+        <f t="shared" si="20"/>
         <v>20</v>
       </c>
       <c r="Z5" s="8">
-        <f t="shared" si="23"/>
+        <f t="shared" si="20"/>
         <v>21</v>
       </c>
       <c r="AA5" s="8">
-        <f t="shared" si="23"/>
+        <f t="shared" si="20"/>
         <v>22</v>
       </c>
     </row>
@@ -4375,17 +4373,17 @@
         <v>67</v>
       </c>
       <c r="E6" s="9">
-        <f t="shared" ref="E6:E42" si="24">ROW(D6)-ROW($E$5)</f>
+        <f t="shared" ref="E6:E42" si="21">ROW(D6)-ROW($E$5)</f>
         <v>1</v>
       </c>
       <c r="F6" s="69">
         <v>1</v>
       </c>
       <c r="G6" s="69" t="s">
+        <v>272</v>
+      </c>
+      <c r="H6" s="69" t="s">
         <v>273</v>
-      </c>
-      <c r="H6" s="69" t="s">
-        <v>274</v>
       </c>
       <c r="I6" s="69" t="s">
         <v>76</v>
@@ -4458,17 +4456,17 @@
         <v>82</v>
       </c>
       <c r="E7" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>2</v>
       </c>
       <c r="F7" s="69">
         <v>1</v>
       </c>
       <c r="G7" s="69" t="s">
+        <v>272</v>
+      </c>
+      <c r="H7" s="69" t="s">
         <v>273</v>
-      </c>
-      <c r="H7" s="69" t="s">
-        <v>274</v>
       </c>
       <c r="I7" s="69" t="s">
         <v>77</v>
@@ -4539,20 +4537,20 @@
         <v>135</v>
       </c>
       <c r="D8" s="68" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E8" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>3</v>
       </c>
       <c r="F8" s="69">
         <v>1</v>
       </c>
       <c r="G8" s="69" t="s">
+        <v>274</v>
+      </c>
+      <c r="H8" s="69" t="s">
         <v>275</v>
-      </c>
-      <c r="H8" s="69" t="s">
-        <v>276</v>
       </c>
       <c r="I8" s="69" t="s">
         <v>88</v>
@@ -4624,20 +4622,20 @@
         <v>135</v>
       </c>
       <c r="D9" s="78" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E9" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>4</v>
       </c>
       <c r="F9" s="79">
         <v>1</v>
       </c>
       <c r="G9" s="79" t="s">
+        <v>276</v>
+      </c>
+      <c r="H9" s="79" t="s">
         <v>277</v>
-      </c>
-      <c r="H9" s="79" t="s">
-        <v>278</v>
       </c>
       <c r="I9" s="79" t="s">
         <v>78</v>
@@ -4698,7 +4696,7 @@
         <v>0</v>
       </c>
       <c r="AA9" s="95">
-        <f t="shared" ref="AA9:AA10" si="25">1/11.3</f>
+        <f t="shared" ref="AA9:AA10" si="22">1/11.3</f>
         <v>8.8495575221238937E-2</v>
       </c>
     </row>
@@ -4711,7 +4709,7 @@
         <v>135</v>
       </c>
       <c r="D10" s="78" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E10" s="9">
         <f>ROW(D10)-ROW($E$5)</f>
@@ -4721,10 +4719,10 @@
         <v>1</v>
       </c>
       <c r="G10" s="79" t="s">
+        <v>276</v>
+      </c>
+      <c r="H10" s="79" t="s">
         <v>277</v>
-      </c>
-      <c r="H10" s="79" t="s">
-        <v>278</v>
       </c>
       <c r="I10" s="79" t="s">
         <v>79</v>
@@ -4786,7 +4784,7 @@
         <v>0</v>
       </c>
       <c r="AA10" s="95">
-        <f t="shared" si="25"/>
+        <f t="shared" si="22"/>
         <v>8.8495575221238937E-2</v>
       </c>
     </row>
@@ -4799,7 +4797,7 @@
         <v>135</v>
       </c>
       <c r="D11" s="84" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E11" s="9">
         <f>ROW(D11)-ROW($E$5)</f>
@@ -4809,10 +4807,10 @@
         <v>1</v>
       </c>
       <c r="G11" s="85" t="s">
+        <v>264</v>
+      </c>
+      <c r="H11" s="85" t="s">
         <v>265</v>
-      </c>
-      <c r="H11" s="85" t="s">
-        <v>266</v>
       </c>
       <c r="I11" s="85" t="s">
         <v>184</v>
@@ -4883,20 +4881,20 @@
         <v>188</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E12" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>7</v>
       </c>
       <c r="F12" s="2">
         <v>1</v>
       </c>
       <c r="G12" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>271</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>272</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>176</v>
@@ -4969,17 +4967,17 @@
         <v>177</v>
       </c>
       <c r="E13" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>8</v>
       </c>
       <c r="F13" s="99">
         <v>1</v>
       </c>
       <c r="G13" s="99" t="s">
+        <v>264</v>
+      </c>
+      <c r="H13" s="99" t="s">
         <v>265</v>
-      </c>
-      <c r="H13" s="99" t="s">
-        <v>266</v>
       </c>
       <c r="I13" s="99" t="s">
         <v>80</v>
@@ -5004,7 +5002,7 @@
         <v>20000</v>
       </c>
       <c r="P13" s="100">
-        <f t="shared" ref="P13:P14" si="26">(1/9)*0.8</f>
+        <f t="shared" ref="P13:P14" si="23">(1/9)*0.8</f>
         <v>8.8888888888888892E-2</v>
       </c>
       <c r="Q13" s="100">
@@ -5039,7 +5037,7 @@
         <v>0</v>
       </c>
       <c r="AA13" s="103">
-        <f t="shared" ref="AA13:AA14" si="27">1/11.3</f>
+        <f t="shared" ref="AA13:AA14" si="24">1/11.3</f>
         <v>8.8495575221238937E-2</v>
       </c>
     </row>
@@ -5055,17 +5053,17 @@
         <v>180</v>
       </c>
       <c r="E14" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>9</v>
       </c>
       <c r="F14" s="107">
         <v>1</v>
       </c>
       <c r="G14" s="107" t="s">
+        <v>264</v>
+      </c>
+      <c r="H14" s="107" t="s">
         <v>265</v>
-      </c>
-      <c r="H14" s="107" t="s">
-        <v>266</v>
       </c>
       <c r="I14" s="107" t="s">
         <v>181</v>
@@ -5091,7 +5089,7 @@
         <v>20000</v>
       </c>
       <c r="P14" s="108">
-        <f t="shared" si="26"/>
+        <f t="shared" si="23"/>
         <v>8.8888888888888892E-2</v>
       </c>
       <c r="Q14" s="108">
@@ -5126,7 +5124,7 @@
         <v>0</v>
       </c>
       <c r="AA14" s="112">
-        <f t="shared" si="27"/>
+        <f t="shared" si="24"/>
         <v>8.8495575221238937E-2</v>
       </c>
     </row>
@@ -5142,17 +5140,17 @@
         <v>65</v>
       </c>
       <c r="E15" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>10</v>
       </c>
       <c r="F15" s="2">
         <v>1</v>
       </c>
       <c r="G15" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="H15" s="2" t="s">
         <v>265</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>266</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>66</v>
@@ -5225,17 +5223,17 @@
         <v>29</v>
       </c>
       <c r="E16" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>11</v>
       </c>
       <c r="F16" s="2">
         <v>1</v>
       </c>
       <c r="G16" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="H16" s="2" t="s">
         <v>265</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>266</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>18</v>
@@ -5305,20 +5303,20 @@
         <v>188</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E17" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>12</v>
       </c>
       <c r="F17" s="2">
         <v>1</v>
       </c>
       <c r="G17" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="H17" s="2" t="s">
         <v>265</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>266</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>185</v>
@@ -5391,17 +5389,17 @@
         <v>30</v>
       </c>
       <c r="E18" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>13</v>
       </c>
       <c r="F18" s="92">
         <v>1</v>
       </c>
       <c r="G18" s="92" t="s">
+        <v>266</v>
+      </c>
+      <c r="H18" s="92" t="s">
         <v>267</v>
-      </c>
-      <c r="H18" s="92" t="s">
-        <v>268</v>
       </c>
       <c r="I18" s="92" t="s">
         <v>19</v>
@@ -5468,23 +5466,23 @@
         <v>27</v>
       </c>
       <c r="C19" s="132" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D19" s="91" t="s">
         <v>31</v>
       </c>
       <c r="E19" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>14</v>
       </c>
       <c r="F19" s="92">
         <v>1</v>
       </c>
       <c r="G19" s="92" t="s">
+        <v>266</v>
+      </c>
+      <c r="H19" s="92" t="s">
         <v>267</v>
-      </c>
-      <c r="H19" s="92" t="s">
-        <v>268</v>
       </c>
       <c r="I19" s="92" t="s">
         <v>20</v>
@@ -5551,23 +5549,23 @@
         <v>111</v>
       </c>
       <c r="C20" s="132" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D20" s="91" t="s">
         <v>32</v>
       </c>
       <c r="E20" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>15</v>
       </c>
       <c r="F20" s="92">
         <v>1</v>
       </c>
       <c r="G20" s="92" t="s">
+        <v>268</v>
+      </c>
+      <c r="H20" s="92" t="s">
         <v>269</v>
-      </c>
-      <c r="H20" s="92" t="s">
-        <v>270</v>
       </c>
       <c r="I20" s="92" t="s">
         <v>13</v>
@@ -5638,20 +5636,20 @@
         <v>188</v>
       </c>
       <c r="D21" s="117" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E21" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>16</v>
       </c>
       <c r="F21" s="62">
         <v>1</v>
       </c>
       <c r="G21" s="62" t="s">
+        <v>264</v>
+      </c>
+      <c r="H21" s="62" t="s">
         <v>265</v>
-      </c>
-      <c r="H21" s="62" t="s">
-        <v>266</v>
       </c>
       <c r="I21" s="62" t="s">
         <v>129</v>
@@ -5720,20 +5718,20 @@
         <v>188</v>
       </c>
       <c r="D22" s="117" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E22" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>17</v>
       </c>
       <c r="F22" s="62">
         <v>1</v>
       </c>
       <c r="G22" s="62" t="s">
+        <v>264</v>
+      </c>
+      <c r="H22" s="62" t="s">
         <v>265</v>
-      </c>
-      <c r="H22" s="62" t="s">
-        <v>266</v>
       </c>
       <c r="I22" s="62" t="s">
         <v>130</v>
@@ -5802,20 +5800,20 @@
         <v>188</v>
       </c>
       <c r="D23" s="120" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E23" s="116">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>18</v>
       </c>
       <c r="F23" s="121">
         <v>1</v>
       </c>
       <c r="G23" s="121" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="H23" s="121" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I23" s="121" t="s">
         <v>131</v>
@@ -5890,17 +5888,17 @@
         <v>37</v>
       </c>
       <c r="E24" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>19</v>
       </c>
       <c r="F24" s="2">
         <v>1</v>
       </c>
       <c r="G24" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H24" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>38</v>
@@ -5979,10 +5977,10 @@
         <v>1</v>
       </c>
       <c r="G25" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H25" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>40</v>
@@ -6003,7 +6001,7 @@
         <v>0</v>
       </c>
       <c r="O25">
-        <f t="shared" ref="O25:O38" si="28">$O$24</f>
+        <f t="shared" ref="O25:O38" si="25">$O$24</f>
         <v>2000000</v>
       </c>
       <c r="P25" s="10">
@@ -6056,17 +6054,17 @@
         <v>132</v>
       </c>
       <c r="E26" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>21</v>
       </c>
       <c r="F26" s="2">
         <v>1</v>
       </c>
       <c r="G26" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H26" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>43</v>
@@ -6087,7 +6085,7 @@
         <v>0</v>
       </c>
       <c r="O26">
-        <f t="shared" si="28"/>
+        <f t="shared" si="25"/>
         <v>2000000</v>
       </c>
       <c r="P26" s="10">
@@ -6130,7 +6128,7 @@
     <row r="27" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A27" s="136"/>
       <c r="B27" s="12" t="str">
-        <f t="shared" ref="B27:B37" si="29">CONCATENATE("RPU_"&amp;D27)</f>
+        <f t="shared" ref="B27:B37" si="26">CONCATENATE("RPU_"&amp;D27)</f>
         <v>RPU_ON_SP198-HH150</v>
       </c>
       <c r="C27" s="11" t="s">
@@ -6140,17 +6138,17 @@
         <v>44</v>
       </c>
       <c r="E27" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>22</v>
       </c>
       <c r="F27" s="2">
         <v>1</v>
       </c>
       <c r="G27" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H27" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>45</v>
@@ -6171,7 +6169,7 @@
         <v>0</v>
       </c>
       <c r="O27">
-        <f t="shared" si="28"/>
+        <f t="shared" si="25"/>
         <v>2000000</v>
       </c>
       <c r="P27" s="10">
@@ -6214,7 +6212,7 @@
     <row r="28" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A28" s="136"/>
       <c r="B28" s="12" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="26"/>
         <v>RPU_ON_SP237-HH100</v>
       </c>
       <c r="C28" s="11" t="s">
@@ -6224,17 +6222,17 @@
         <v>46</v>
       </c>
       <c r="E28" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>23</v>
       </c>
       <c r="F28" s="2">
         <v>1</v>
       </c>
       <c r="G28" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H28" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>47</v>
@@ -6255,7 +6253,7 @@
         <v>0</v>
       </c>
       <c r="O28">
-        <f t="shared" si="28"/>
+        <f t="shared" si="25"/>
         <v>2000000</v>
       </c>
       <c r="P28" s="10">
@@ -6298,7 +6296,7 @@
     <row r="29" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A29" s="136"/>
       <c r="B29" s="12" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="26"/>
         <v>RPU_ON_SP237-HH150</v>
       </c>
       <c r="C29" s="11" t="s">
@@ -6308,17 +6306,17 @@
         <v>48</v>
       </c>
       <c r="E29" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>24</v>
       </c>
       <c r="F29" s="2">
         <v>1</v>
       </c>
       <c r="G29" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H29" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H29" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>49</v>
@@ -6339,7 +6337,7 @@
         <v>0</v>
       </c>
       <c r="O29">
-        <f t="shared" si="28"/>
+        <f t="shared" si="25"/>
         <v>2000000</v>
       </c>
       <c r="P29" s="10">
@@ -6382,7 +6380,7 @@
     <row r="30" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A30" s="136"/>
       <c r="B30" s="12" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="26"/>
         <v>RPU_ON_SP277-HH100</v>
       </c>
       <c r="C30" s="11" t="s">
@@ -6392,17 +6390,17 @@
         <v>50</v>
       </c>
       <c r="E30" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>25</v>
       </c>
       <c r="F30" s="2">
         <v>1</v>
       </c>
       <c r="G30" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H30" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>51</v>
@@ -6423,7 +6421,7 @@
         <v>0</v>
       </c>
       <c r="O30">
-        <f t="shared" si="28"/>
+        <f t="shared" si="25"/>
         <v>2000000</v>
       </c>
       <c r="P30" s="10">
@@ -6466,7 +6464,7 @@
     <row r="31" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A31" s="136"/>
       <c r="B31" s="12" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="26"/>
         <v>RPU_ON_SP277-HH150</v>
       </c>
       <c r="C31" s="11" t="s">
@@ -6476,17 +6474,17 @@
         <v>52</v>
       </c>
       <c r="E31" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>26</v>
       </c>
       <c r="F31" s="2">
         <v>1</v>
       </c>
       <c r="G31" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I31" s="2" t="s">
         <v>53</v>
@@ -6507,7 +6505,7 @@
         <v>0</v>
       </c>
       <c r="O31">
-        <f t="shared" si="28"/>
+        <f t="shared" si="25"/>
         <v>2000000</v>
       </c>
       <c r="P31" s="10">
@@ -6550,7 +6548,7 @@
     <row r="32" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A32" s="136"/>
       <c r="B32" s="12" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="26"/>
         <v>RPU_ON_SP321-HH100</v>
       </c>
       <c r="C32" s="11" t="s">
@@ -6560,17 +6558,17 @@
         <v>54</v>
       </c>
       <c r="E32" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>27</v>
       </c>
       <c r="F32" s="2">
         <v>1</v>
       </c>
       <c r="G32" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H32" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I32" s="2" t="s">
         <v>55</v>
@@ -6591,7 +6589,7 @@
         <v>0</v>
       </c>
       <c r="O32">
-        <f t="shared" si="28"/>
+        <f t="shared" si="25"/>
         <v>2000000</v>
       </c>
       <c r="P32" s="10">
@@ -6634,7 +6632,7 @@
     <row r="33" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A33" s="136"/>
       <c r="B33" s="12" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="26"/>
         <v>RPU_ON_SP321-HH150</v>
       </c>
       <c r="C33" s="11" t="s">
@@ -6644,17 +6642,17 @@
         <v>56</v>
       </c>
       <c r="E33" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>28</v>
       </c>
       <c r="F33" s="2">
         <v>1</v>
       </c>
       <c r="G33" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H33" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I33" s="2" t="s">
         <v>57</v>
@@ -6675,7 +6673,7 @@
         <v>0</v>
       </c>
       <c r="O33">
-        <f t="shared" si="28"/>
+        <f t="shared" si="25"/>
         <v>2000000</v>
       </c>
       <c r="P33" s="10">
@@ -6718,7 +6716,7 @@
     <row r="34" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A34" s="136"/>
       <c r="B34" s="12" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="26"/>
         <v>RPU_OFF_SP379-HH100</v>
       </c>
       <c r="C34" s="11" t="s">
@@ -6728,17 +6726,17 @@
         <v>58</v>
       </c>
       <c r="E34" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>29</v>
       </c>
       <c r="F34" s="2">
         <v>1</v>
       </c>
       <c r="G34" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H34" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I34" s="2" t="s">
         <v>59</v>
@@ -6759,7 +6757,7 @@
         <v>0</v>
       </c>
       <c r="O34">
-        <f t="shared" si="28"/>
+        <f t="shared" si="25"/>
         <v>2000000</v>
       </c>
       <c r="P34" s="10">
@@ -6802,7 +6800,7 @@
     <row r="35" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A35" s="136"/>
       <c r="B35" s="12" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="26"/>
         <v>RPU_OFF_SP379-HH150</v>
       </c>
       <c r="C35" s="11" t="s">
@@ -6812,17 +6810,17 @@
         <v>60</v>
       </c>
       <c r="E35" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>30</v>
       </c>
       <c r="F35" s="2">
         <v>1</v>
       </c>
       <c r="G35" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H35" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H35" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I35" s="2" t="s">
         <v>61</v>
@@ -6843,7 +6841,7 @@
         <v>0</v>
       </c>
       <c r="O35">
-        <f t="shared" si="28"/>
+        <f t="shared" si="25"/>
         <v>2000000</v>
       </c>
       <c r="P35" s="10">
@@ -6886,7 +6884,7 @@
     <row r="36" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A36" s="136"/>
       <c r="B36" s="12" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="26"/>
         <v>RPU_OFF_SP450-HH100</v>
       </c>
       <c r="C36" s="11" t="s">
@@ -6896,17 +6894,17 @@
         <v>62</v>
       </c>
       <c r="E36" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>31</v>
       </c>
       <c r="F36" s="2">
         <v>1</v>
       </c>
       <c r="G36" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H36" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I36" s="2" t="s">
         <v>63</v>
@@ -6927,7 +6925,7 @@
         <v>0</v>
       </c>
       <c r="O36">
-        <f t="shared" si="28"/>
+        <f t="shared" si="25"/>
         <v>2000000</v>
       </c>
       <c r="P36" s="10">
@@ -6970,7 +6968,7 @@
     <row r="37" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A37" s="136"/>
       <c r="B37" s="12" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="26"/>
         <v>RPU_OFF_SP450-HH150</v>
       </c>
       <c r="C37" s="11" t="s">
@@ -6980,17 +6978,17 @@
         <v>133</v>
       </c>
       <c r="E37" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>32</v>
       </c>
       <c r="F37" s="2">
         <v>1</v>
       </c>
       <c r="G37" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H37" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I37" s="2" t="s">
         <v>64</v>
@@ -7011,7 +7009,7 @@
         <v>0</v>
       </c>
       <c r="O37">
-        <f t="shared" si="28"/>
+        <f t="shared" si="25"/>
         <v>2000000</v>
       </c>
       <c r="P37" s="10">
@@ -7063,17 +7061,17 @@
         <v>33</v>
       </c>
       <c r="E38" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>33</v>
       </c>
       <c r="F38" s="2">
         <v>1</v>
       </c>
       <c r="G38" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H38" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I38" s="2" t="s">
         <v>21</v>
@@ -7094,7 +7092,7 @@
         <v>0</v>
       </c>
       <c r="O38">
-        <f t="shared" si="28"/>
+        <f t="shared" si="25"/>
         <v>2000000</v>
       </c>
       <c r="P38" s="10">
@@ -7146,17 +7144,17 @@
         <v>189</v>
       </c>
       <c r="E39" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>34</v>
       </c>
       <c r="F39" s="2">
         <v>1</v>
       </c>
       <c r="G39" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H39" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>189</v>
@@ -7228,17 +7226,17 @@
         <v>34</v>
       </c>
       <c r="E40" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>35</v>
       </c>
       <c r="F40" s="2">
         <v>1</v>
       </c>
       <c r="G40" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H40" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H40" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>22</v>
@@ -7311,17 +7309,17 @@
         <v>35</v>
       </c>
       <c r="E41" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>36</v>
       </c>
       <c r="F41" s="2">
         <v>1</v>
       </c>
       <c r="G41" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H41" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>264</v>
       </c>
       <c r="I41" s="2" t="s">
         <v>23</v>
@@ -7394,17 +7392,17 @@
         <v>36</v>
       </c>
       <c r="E42" s="9">
-        <f t="shared" si="24"/>
+        <f t="shared" si="21"/>
         <v>37</v>
       </c>
       <c r="F42" s="2">
         <v>1</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="I42" s="2" t="s">
         <v>24</v>
@@ -9184,7 +9182,7 @@
     </row>
     <row r="2" spans="1:140" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4" spans="1:140" s="16" customFormat="1" x14ac:dyDescent="0.35">
@@ -9756,7 +9754,7 @@
         <v>171</v>
       </c>
       <c r="C6" s="42" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D6" s="42" t="str">
         <f>Data_base_case!$R$1</f>
@@ -9782,7 +9780,7 @@
         <v>171</v>
       </c>
       <c r="C7" s="42" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D7" s="42" t="str">
         <f>Data_base_case!$R$1</f>
@@ -9837,7 +9835,7 @@
         <v>136</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D9" s="29" t="str">
         <f>Data_base_case!$R$1</f>
@@ -9863,7 +9861,7 @@
         <v>136</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D10" s="29" t="str">
         <f>Data_base_case!$R$1</f>
@@ -9888,7 +9886,7 @@
         <v>125</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D11" s="23" t="str">
         <f>Data_base_case!$R$1</f>
@@ -9914,7 +9912,7 @@
         <v>125</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D12" s="23" t="str">
         <f>Data_base_case!$R$1</f>
@@ -9942,7 +9940,7 @@
         <v>172</v>
       </c>
       <c r="C13" s="44" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D13" s="44" t="str">
         <f>Data_base_case!$R$1</f>
@@ -9967,7 +9965,7 @@
         <v>172</v>
       </c>
       <c r="C14" s="44" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D14" s="44" t="str">
         <f>Data_base_case!$R$1</f>
@@ -10037,7 +10035,7 @@
         <v>128</v>
       </c>
       <c r="C2" s="141" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>186</v>
@@ -10187,7 +10185,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C8" s="14" t="s">
         <v>124</v>
@@ -10215,7 +10213,7 @@
         <v>175</v>
       </c>
       <c r="K8" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L8" t="b">
         <v>0</v>
@@ -10242,7 +10240,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C9" s="14" t="s">
         <v>124</v>
@@ -10270,7 +10268,7 @@
         <v>175</v>
       </c>
       <c r="K9" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L9" t="b">
         <v>0</v>
@@ -10297,7 +10295,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C10" s="14" t="s">
         <v>124</v>
@@ -10325,7 +10323,7 @@
         <v>175</v>
       </c>
       <c r="K10" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L10" t="b">
         <v>0</v>
@@ -10352,7 +10350,7 @@
         <v>4</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C11" s="14" t="s">
         <v>170</v>
@@ -10380,7 +10378,7 @@
         <v>175</v>
       </c>
       <c r="K11" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L11" t="b">
         <v>0</v>
@@ -10407,7 +10405,7 @@
         <v>5</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C12" s="14" t="s">
         <v>170</v>
@@ -10435,7 +10433,7 @@
         <v>175</v>
       </c>
       <c r="K12" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L12" t="b">
         <v>0</v>
@@ -10462,7 +10460,7 @@
         <v>6</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C13" s="14" t="s">
         <v>170</v>
@@ -10490,7 +10488,7 @@
         <v>175</v>
       </c>
       <c r="K13" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L13" t="b">
         <v>0</v>
@@ -10517,7 +10515,7 @@
         <v>7</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C14" s="14" t="s">
         <v>170</v>
@@ -10545,7 +10543,7 @@
         <v>175</v>
       </c>
       <c r="K14" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L14" t="b">
         <v>0</v>
@@ -10572,7 +10570,7 @@
         <v>8</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C15" s="14" t="s">
         <v>170</v>
@@ -10600,7 +10598,7 @@
         <v>175</v>
       </c>
       <c r="K15" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L15" t="b">
         <v>0</v>
@@ -10627,7 +10625,7 @@
         <v>9</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C16" s="14" t="s">
         <v>170</v>
@@ -10655,7 +10653,7 @@
         <v>175</v>
       </c>
       <c r="K16" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L16" t="b">
         <v>0</v>
@@ -10682,7 +10680,7 @@
         <v>10</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C17" s="14" t="s">
         <v>170</v>
@@ -10710,7 +10708,7 @@
         <v>175</v>
       </c>
       <c r="K17" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L17" t="b">
         <v>0</v>
@@ -10737,7 +10735,7 @@
         <v>11</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C18" s="14" t="s">
         <v>170</v>
@@ -10765,7 +10763,7 @@
         <v>175</v>
       </c>
       <c r="K18" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L18" t="b">
         <v>0</v>
@@ -10792,7 +10790,7 @@
         <v>12</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C19" s="14" t="s">
         <v>170</v>
@@ -10820,7 +10818,7 @@
         <v>175</v>
       </c>
       <c r="K19" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L19" t="b">
         <v>0</v>
@@ -10847,7 +10845,7 @@
         <v>13</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C20" s="14" t="s">
         <v>136</v>
@@ -10875,7 +10873,7 @@
         <v>175</v>
       </c>
       <c r="K20" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L20" t="b">
         <v>0</v>
@@ -10902,7 +10900,7 @@
         <v>14</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C21" s="14" t="s">
         <v>136</v>
@@ -10930,7 +10928,7 @@
         <v>175</v>
       </c>
       <c r="K21" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L21" t="b">
         <v>0</v>
@@ -10957,7 +10955,7 @@
         <v>15</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C22" s="14" t="s">
         <v>136</v>
@@ -10985,7 +10983,7 @@
         <v>175</v>
       </c>
       <c r="K22" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L22" t="b">
         <v>0</v>
@@ -11012,7 +11010,7 @@
         <v>16</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C23" s="14" t="s">
         <v>125</v>
@@ -11040,7 +11038,7 @@
         <v>175</v>
       </c>
       <c r="K23" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L23" t="b">
         <v>0</v>
@@ -11067,7 +11065,7 @@
         <v>17</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C24" s="14" t="s">
         <v>125</v>
@@ -11095,7 +11093,7 @@
         <v>175</v>
       </c>
       <c r="K24" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L24" t="b">
         <v>0</v>
@@ -11122,7 +11120,7 @@
         <v>18</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C25" s="14" t="s">
         <v>125</v>
@@ -11150,7 +11148,7 @@
         <v>175</v>
       </c>
       <c r="K25" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L25" t="b">
         <v>0</v>
@@ -11177,7 +11175,7 @@
         <v>19</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C26" s="14" t="s">
         <v>172</v>
@@ -11205,7 +11203,7 @@
         <v>175</v>
       </c>
       <c r="K26" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L26" t="b">
         <v>0</v>
@@ -11232,7 +11230,7 @@
         <v>20</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C27" s="14" t="s">
         <v>172</v>
@@ -11260,7 +11258,7 @@
         <v>175</v>
       </c>
       <c r="K27" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L27" t="b">
         <v>0</v>
@@ -11287,7 +11285,7 @@
         <v>21</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C28" s="14" t="s">
         <v>172</v>
@@ -11315,7 +11313,7 @@
         <v>175</v>
       </c>
       <c r="K28" s="17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L28" t="b">
         <v>0</v>
@@ -11403,7 +11401,7 @@
         <v>190</v>
       </c>
       <c r="C2" s="54" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D2" s="54">
         <v>2023</v>

</xml_diff>